<commit_message>
Updated new coding for prerelease data
</commit_message>
<xml_diff>
--- a/Outputs&ExcelFiles/RegressionOutput/regression_results.xlsx
+++ b/Outputs&ExcelFiles/RegressionOutput/regression_results.xlsx
@@ -464,32 +464,32 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>15.624***</t>
+          <t>15.972***</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>11.682***</t>
+          <t>11.754***</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>8.493***</t>
+          <t>7.735***</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>6.568***</t>
+          <t>5.036***</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>9.603***</t>
+          <t>9.361***</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>8.680***</t>
+          <t>8.006***</t>
         </is>
       </c>
     </row>
@@ -497,64 +497,64 @@
       <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>(0.103)</t>
+          <t>(0.188)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>(0.264)</t>
+          <t>(0.472)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>(0.607)</t>
+          <t>(1.671)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>(0.723)</t>
+          <t>(1.610)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>(0.746)</t>
+          <t>(2.074)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>(0.620)</t>
+          <t>(1.728)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tomatometer</t>
+          <t>PreRelease Tomatometer</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.015***</t>
+          <t>0.012***</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.001</t>
+          <t>-0.000</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.004***</t>
+          <t>0.005*</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.007***</t>
+          <t>0.008***</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.002</t>
+          <t>0.004</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -567,32 +567,32 @@
       <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
-          <t>(0.002)</t>
+          <t>(0.003)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>(0.002)</t>
+          <t>(0.003)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>(0.002)</t>
+          <t>(0.003)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>(0.002)</t>
+          <t>(0.003)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>(0.002)</t>
+          <t>(0.004)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>(0.002)</t>
+          <t>(0.004)</t>
         </is>
       </c>
     </row>
@@ -605,27 +605,27 @@
       <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.922***</t>
+          <t>1.147***</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.478***</t>
+          <t>0.440***</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.332**</t>
+          <t>0.347**</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0.514***</t>
+          <t>0.368*</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>0.485***</t>
+          <t>0.432***</t>
         </is>
       </c>
     </row>
@@ -634,27 +634,27 @@
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
-          <t>(0.059)</t>
+          <t>(0.121)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>(0.089)</t>
+          <t>(0.155)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>(0.151)</t>
+          <t>(0.139)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>(0.098)</t>
+          <t>(0.205)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>(0.089)</t>
+          <t>(0.152)</t>
         </is>
       </c>
     </row>
@@ -668,14 +668,14 @@
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.813***</t>
+          <t>0.811***</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>0.563***</t>
+          <t>0.503**</t>
         </is>
       </c>
     </row>
@@ -685,14 +685,14 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>(0.065)</t>
+          <t>(0.122)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>(0.143)</t>
+          <t>(0.237)</t>
         </is>
       </c>
     </row>
@@ -706,22 +706,22 @@
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.294***</t>
+          <t>0.372***</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0.484***</t>
+          <t>0.578***</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0.223***</t>
+          <t>0.300**</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>0.286***</t>
+          <t>0.365***</t>
         </is>
       </c>
     </row>
@@ -731,22 +731,22 @@
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>(0.048)</t>
+          <t>(0.116)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>(0.061)</t>
+          <t>(0.109)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>(0.057)</t>
+          <t>(0.134)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>(0.048)</t>
+          <t>(0.116)</t>
         </is>
       </c>
     </row>
@@ -760,22 +760,22 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>-0.034</t>
+          <t>-0.053</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>-0.048</t>
+          <t>-0.059</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>-0.023</t>
+          <t>-0.059</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>-0.033</t>
+          <t>-0.049</t>
         </is>
       </c>
     </row>
@@ -785,29 +785,29 @@
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>(0.023)</t>
+          <t>(0.035)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>(0.034)</t>
+          <t>(0.043)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>(0.030)</t>
+          <t>(0.051)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>(0.023)</t>
+          <t>(0.035)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Tomatometer_Franchise</t>
+          <t>PreRelease_Tomatometer_Franchise</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -817,7 +817,7 @@
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>0.005**</t>
+          <t>0.005</t>
         </is>
       </c>
     </row>
@@ -830,7 +830,7 @@
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>(0.002)</t>
+          <t>(0.004)</t>
         </is>
       </c>
     </row>
@@ -842,32 +842,32 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0.116</t>
+          <t>0.076</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.398</t>
+          <t>0.353</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.603</t>
+          <t>0.616</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0.682</t>
+          <t>0.695</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>0.369</t>
+          <t>0.227</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>0.606</t>
+          <t>0.619</t>
         </is>
       </c>
     </row>
@@ -879,32 +879,32 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0.114</t>
+          <t>0.071</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.396</t>
+          <t>0.347</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.600</t>
+          <t>0.607</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0.674</t>
+          <t>0.679</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0.362</t>
+          <t>0.202</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>0.601</t>
+          <t>0.608</t>
         </is>
       </c>
     </row>
@@ -916,32 +916,32 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0.114</t>
+          <t>0.071</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.396</t>
+          <t>0.347</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.600</t>
+          <t>0.607</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0.674</t>
+          <t>0.679</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0.362</t>
+          <t>0.202</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>0.601</t>
+          <t>0.608</t>
         </is>
       </c>
     </row>
@@ -953,32 +953,32 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>532</t>
+          <t>212</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>532</t>
+          <t>212</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>532</t>
+          <t>212</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>164</t>
+          <t>81</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>368</t>
+          <t>131</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>532</t>
+          <t>212</t>
         </is>
       </c>
     </row>
@@ -1025,13 +1025,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>532</v>
+        <v>212</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1159</v>
+        <v>0.07580000000000001</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1142</v>
+        <v>0.07140000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -1041,13 +1041,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>532</v>
+        <v>212</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3982</v>
+        <v>0.3535</v>
       </c>
       <c r="D3" t="n">
-        <v>0.3959</v>
+        <v>0.3473</v>
       </c>
     </row>
     <row r="4">
@@ -1057,13 +1057,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>532</v>
+        <v>212</v>
       </c>
       <c r="C4" t="n">
-        <v>0.6032999999999999</v>
+        <v>0.616</v>
       </c>
       <c r="D4" t="n">
-        <v>0.5996</v>
+        <v>0.6066</v>
       </c>
     </row>
     <row r="5">
@@ -1073,13 +1073,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>164</v>
+        <v>81</v>
       </c>
       <c r="C5" t="n">
-        <v>0.6820000000000001</v>
+        <v>0.6952</v>
       </c>
       <c r="D5" t="n">
-        <v>0.674</v>
+        <v>0.6791</v>
       </c>
     </row>
     <row r="6">
@@ -1089,13 +1089,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>368</v>
+        <v>131</v>
       </c>
       <c r="C6" t="n">
-        <v>0.3688</v>
+        <v>0.227</v>
       </c>
       <c r="D6" t="n">
-        <v>0.3618</v>
+        <v>0.2025</v>
       </c>
     </row>
     <row r="7">
@@ -1105,13 +1105,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>532</v>
+        <v>212</v>
       </c>
       <c r="C7" t="n">
-        <v>0.606</v>
+        <v>0.6194</v>
       </c>
       <c r="D7" t="n">
-        <v>0.6015</v>
+        <v>0.6082</v>
       </c>
     </row>
   </sheetData>
@@ -1143,11 +1143,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tomatometer</t>
+          <t>PreRelease Tomatometer</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1.405927331639062</v>
+        <v>1.440491849152871</v>
       </c>
     </row>
     <row r="3">
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2.023350181034979</v>
+        <v>1.939093343925006</v>
       </c>
     </row>
     <row r="4">
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.191191049764012</v>
+        <v>1.364662396552164</v>
       </c>
     </row>
     <row r="5">
@@ -1177,7 +1177,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1.704211564257394</v>
+        <v>1.749735948338289</v>
       </c>
     </row>
     <row r="6">
@@ -1187,7 +1187,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1.021781470955481</v>
+        <v>1.11966099944044</v>
       </c>
     </row>
   </sheetData>
@@ -1258,22 +1258,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>15.62365261155204</v>
+        <v>15.97209917541096</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1025234193923273</v>
+        <v>0.1878966559657819</v>
       </c>
       <c r="E2" t="n">
-        <v>152.3910605416394</v>
+        <v>85.00470161810469</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>1.230542205178987e-164</v>
       </c>
       <c r="G2" t="n">
-        <v>15.42225047691931</v>
+        <v>15.60169383893811</v>
       </c>
       <c r="H2" t="n">
-        <v>15.82505474618476</v>
+        <v>16.34250451188382</v>
       </c>
     </row>
     <row r="3">
@@ -1284,26 +1284,26 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tomatometer</t>
+          <t>PreRelease Tomatometer</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.01460379724967668</v>
+        <v>0.01201470676455575</v>
       </c>
       <c r="D3" t="n">
-        <v>0.001752218551364059</v>
+        <v>0.002895465559289128</v>
       </c>
       <c r="E3" t="n">
-        <v>8.334461039867417</v>
+        <v>4.14949047693232</v>
       </c>
       <c r="F3" t="n">
-        <v>6.723699330039021e-16</v>
+        <v>4.840299382119782e-05</v>
       </c>
       <c r="G3" t="n">
-        <v>0.01116165145821279</v>
+        <v>0.006306803719546923</v>
       </c>
       <c r="H3" t="n">
-        <v>0.01804594304114056</v>
+        <v>0.01772260980956458</v>
       </c>
     </row>
   </sheetData>
@@ -1374,22 +1374,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>11.68178651045915</v>
+        <v>11.75426494946652</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2641700716289256</v>
+        <v>0.4722143907894881</v>
       </c>
       <c r="E2" t="n">
-        <v>44.22070387620717</v>
+        <v>24.89179740967814</v>
       </c>
       <c r="F2" t="n">
-        <v>8.062016887041255e-180</v>
+        <v>1.958519354661283e-64</v>
       </c>
       <c r="G2" t="n">
-        <v>11.16283535919681</v>
+        <v>10.82335119801694</v>
       </c>
       <c r="H2" t="n">
-        <v>12.2007376617215</v>
+        <v>12.6851787009161</v>
       </c>
     </row>
     <row r="3">
@@ -1400,26 +1400,26 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tomatometer</t>
+          <t>PreRelease Tomatometer</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.001040560587293203</v>
+        <v>-0.0004983840935438317</v>
       </c>
       <c r="D3" t="n">
-        <v>0.001683808451304955</v>
+        <v>0.00276349653570909</v>
       </c>
       <c r="E3" t="n">
-        <v>0.6179803804208054</v>
+        <v>-0.1803454743307469</v>
       </c>
       <c r="F3" t="n">
-        <v>0.5368542242258058</v>
+        <v>0.8570561043948512</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.002267211292094443</v>
+        <v>-0.00594628440609852</v>
       </c>
       <c r="H3" t="n">
-        <v>0.004348332466680848</v>
+        <v>0.004949516219010856</v>
       </c>
     </row>
     <row r="4">
@@ -1434,22 +1434,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.9215380049344202</v>
+        <v>1.147242928971496</v>
       </c>
       <c r="D4" t="n">
-        <v>0.05850044477835517</v>
+        <v>0.1210838323066242</v>
       </c>
       <c r="E4" t="n">
-        <v>15.75266664084209</v>
+        <v>9.474782116792429</v>
       </c>
       <c r="F4" t="n">
-        <v>4.001164030014963e-46</v>
+        <v>6.027324145467443e-18</v>
       </c>
       <c r="G4" t="n">
-        <v>0.8066163070301571</v>
+        <v>0.9085407488367503</v>
       </c>
       <c r="H4" t="n">
-        <v>1.036459702838683</v>
+        <v>1.385945109106242</v>
       </c>
     </row>
   </sheetData>
@@ -1520,22 +1520,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>8.493391910654937</v>
+        <v>7.734831894739729</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6073119760325122</v>
+        <v>1.671458200292565</v>
       </c>
       <c r="E2" t="n">
-        <v>13.98522052231067</v>
+        <v>4.627595170125018</v>
       </c>
       <c r="F2" t="n">
-        <v>1.918811620801304e-44</v>
+        <v>3.699362486727394e-06</v>
       </c>
       <c r="G2" t="n">
-        <v>7.30308231025136</v>
+        <v>4.458834020502167</v>
       </c>
       <c r="H2" t="n">
-        <v>9.683701511058514</v>
+        <v>11.01082976897729</v>
       </c>
     </row>
     <row r="3">
@@ -1546,26 +1546,26 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tomatometer</t>
+          <t>PreRelease Tomatometer</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.004190904439223538</v>
+        <v>0.005048641862816606</v>
       </c>
       <c r="D3" t="n">
-        <v>0.00159865611981058</v>
+        <v>0.002787120150473305</v>
       </c>
       <c r="E3" t="n">
-        <v>2.62151715261948</v>
+        <v>1.811418808751123</v>
       </c>
       <c r="F3" t="n">
-        <v>0.008753935709635516</v>
+        <v>0.07007604663487429</v>
       </c>
       <c r="G3" t="n">
-        <v>0.001057596020730251</v>
+        <v>-0.0004140132526969289</v>
       </c>
       <c r="H3" t="n">
-        <v>0.007324212857716826</v>
+        <v>0.01051129697833014</v>
       </c>
     </row>
     <row r="4">
@@ -1580,22 +1580,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.4783932373928859</v>
+        <v>0.4401876326289644</v>
       </c>
       <c r="D4" t="n">
-        <v>0.08892369421288997</v>
+        <v>0.1550309922677578</v>
       </c>
       <c r="E4" t="n">
-        <v>5.379817399933663</v>
+        <v>2.839352481655447</v>
       </c>
       <c r="F4" t="n">
-        <v>7.456142756623541e-08</v>
+        <v>0.004520519147822474</v>
       </c>
       <c r="G4" t="n">
-        <v>0.3041059993633687</v>
+        <v>0.1363324712966516</v>
       </c>
       <c r="H4" t="n">
-        <v>0.652680475422403</v>
+        <v>0.7440427939612773</v>
       </c>
     </row>
     <row r="5">
@@ -1610,22 +1610,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.8134983044614144</v>
+        <v>0.8113496063989527</v>
       </c>
       <c r="D5" t="n">
-        <v>0.06527355088933294</v>
+        <v>0.1217476622638078</v>
       </c>
       <c r="E5" t="n">
-        <v>12.46290868778761</v>
+        <v>6.664190435467149</v>
       </c>
       <c r="F5" t="n">
-        <v>1.189515188036131e-35</v>
+        <v>2.661282063422886e-11</v>
       </c>
       <c r="G5" t="n">
-        <v>0.6855644955752793</v>
+        <v>0.5727285731599432</v>
       </c>
       <c r="H5" t="n">
-        <v>0.9414321133475494</v>
+        <v>1.049970639637962</v>
       </c>
     </row>
     <row r="6">
@@ -1640,22 +1640,22 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.2944567414181506</v>
+        <v>0.3718041211768801</v>
       </c>
       <c r="D6" t="n">
-        <v>0.04793456288047249</v>
+        <v>0.1159848995270536</v>
       </c>
       <c r="E6" t="n">
-        <v>6.142889884119627</v>
+        <v>3.20562523822471</v>
       </c>
       <c r="F6" t="n">
-        <v>8.103346202796042e-10</v>
+        <v>0.001347693854582435</v>
       </c>
       <c r="G6" t="n">
-        <v>0.200506724557754</v>
+        <v>0.1444778953533584</v>
       </c>
       <c r="H6" t="n">
-        <v>0.3884067582785473</v>
+        <v>0.5991303470004019</v>
       </c>
     </row>
     <row r="7">
@@ -1670,22 +1670,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>-0.03354792235687655</v>
+        <v>-0.05265713472734057</v>
       </c>
       <c r="D7" t="n">
-        <v>0.02347373698555685</v>
+        <v>0.0352318553492896</v>
       </c>
       <c r="E7" t="n">
-        <v>-1.429168367078418</v>
+        <v>-1.494588752289548</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1529558472464817</v>
+        <v>0.1350218033881215</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.0795556014311338</v>
+        <v>-0.121710302320473</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0124597567173807</v>
+        <v>0.0163960328657919</v>
       </c>
     </row>
   </sheetData>
@@ -1756,22 +1756,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6.567583425343081</v>
+        <v>5.036143983321161</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7232702598227061</v>
+        <v>1.609667486153476</v>
       </c>
       <c r="E2" t="n">
-        <v>9.08040021851995</v>
+        <v>3.12868590975626</v>
       </c>
       <c r="F2" t="n">
-        <v>1.081763413227801e-19</v>
+        <v>0.001755898929322412</v>
       </c>
       <c r="G2" t="n">
-        <v>5.14999976500165</v>
+        <v>1.881253683375221</v>
       </c>
       <c r="H2" t="n">
-        <v>7.985167085684512</v>
+        <v>8.191034283267101</v>
       </c>
     </row>
     <row r="3">
@@ -1782,26 +1782,26 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tomatometer</t>
+          <t>PreRelease Tomatometer</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.006961275268506314</v>
+        <v>0.00779379585019752</v>
       </c>
       <c r="D3" t="n">
-        <v>0.002122029533785587</v>
+        <v>0.00256624366064984</v>
       </c>
       <c r="E3" t="n">
-        <v>3.28047991683121</v>
+        <v>3.037044365547084</v>
       </c>
       <c r="F3" t="n">
-        <v>0.001036306424456095</v>
+        <v>0.002389102893998891</v>
       </c>
       <c r="G3" t="n">
-        <v>0.002802173808156241</v>
+        <v>0.002764050699769606</v>
       </c>
       <c r="H3" t="n">
-        <v>0.01112037672885639</v>
+        <v>0.01282354100062543</v>
       </c>
     </row>
     <row r="4">
@@ -1816,22 +1816,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.3319115938018666</v>
+        <v>0.3471413457956581</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1507858956684489</v>
+        <v>0.1392540786580848</v>
       </c>
       <c r="E4" t="n">
-        <v>2.201211143326566</v>
+        <v>2.492863039566733</v>
       </c>
       <c r="F4" t="n">
-        <v>0.02772107979398728</v>
+        <v>0.01267177147037322</v>
       </c>
       <c r="G4" t="n">
-        <v>0.03637666891509272</v>
+        <v>0.0742083669255042</v>
       </c>
       <c r="H4" t="n">
-        <v>0.6274465186886405</v>
+        <v>0.620074324665812</v>
       </c>
     </row>
     <row r="5">
@@ -1846,22 +1846,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.4838306434421289</v>
+        <v>0.5781623369295145</v>
       </c>
       <c r="D5" t="n">
-        <v>0.06091086613830492</v>
+        <v>0.1089108926439173</v>
       </c>
       <c r="E5" t="n">
-        <v>7.943256665297411</v>
+        <v>5.308581381476766</v>
       </c>
       <c r="F5" t="n">
-        <v>1.969408382050885e-15</v>
+        <v>1.104817539371188e-07</v>
       </c>
       <c r="G5" t="n">
-        <v>0.364447539543911</v>
+        <v>0.3647009098233281</v>
       </c>
       <c r="H5" t="n">
-        <v>0.6032137473403468</v>
+        <v>0.7916237640357008</v>
       </c>
     </row>
     <row r="6">
@@ -1876,22 +1876,22 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>-0.04751517896190219</v>
+        <v>-0.05860328903413342</v>
       </c>
       <c r="D6" t="n">
-        <v>0.03396818957447517</v>
+        <v>0.04309162375032128</v>
       </c>
       <c r="E6" t="n">
-        <v>-1.398813995009221</v>
+        <v>-1.359969384623073</v>
       </c>
       <c r="F6" t="n">
-        <v>0.1618687684413951</v>
+        <v>0.173839612319058</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.1140916071479025</v>
+        <v>-0.1430613196201139</v>
       </c>
       <c r="H6" t="n">
-        <v>0.01906124922409809</v>
+        <v>0.0258547415518471</v>
       </c>
     </row>
   </sheetData>
@@ -1962,22 +1962,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>9.602894093670052</v>
+        <v>9.361214516285859</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7459413322921771</v>
+        <v>2.073555562081241</v>
       </c>
       <c r="E2" t="n">
-        <v>12.87352460301624</v>
+        <v>4.514571341840461</v>
       </c>
       <c r="F2" t="n">
-        <v>6.343977326463553e-38</v>
+        <v>6.344496230421915e-06</v>
       </c>
       <c r="G2" t="n">
-        <v>8.140875947797561</v>
+        <v>5.297120294663919</v>
       </c>
       <c r="H2" t="n">
-        <v>11.06491223954254</v>
+        <v>13.4253087379078</v>
       </c>
     </row>
     <row r="3">
@@ -1988,26 +1988,26 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tomatometer</t>
+          <t>PreRelease Tomatometer</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.002416941514476287</v>
+        <v>0.003560925878051683</v>
       </c>
       <c r="D3" t="n">
-        <v>0.002003029361996693</v>
+        <v>0.003970665273319316</v>
       </c>
       <c r="E3" t="n">
-        <v>1.206643077896268</v>
+        <v>0.8968083766665359</v>
       </c>
       <c r="F3" t="n">
-        <v>0.2275696292853787</v>
+        <v>0.3698211773455941</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.001508923895013474</v>
+        <v>-0.004221435052318066</v>
       </c>
       <c r="H3" t="n">
-        <v>0.006342806923966047</v>
+        <v>0.01134328680842143</v>
       </c>
     </row>
     <row r="4">
@@ -2022,22 +2022,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.5135935840324247</v>
+        <v>0.3680825081717264</v>
       </c>
       <c r="D4" t="n">
-        <v>0.09821899639743245</v>
+        <v>0.2053226609704401</v>
       </c>
       <c r="E4" t="n">
-        <v>5.229065688619178</v>
+        <v>1.792702794869382</v>
       </c>
       <c r="F4" t="n">
-        <v>1.703688285318491e-07</v>
+        <v>0.07302045939956175</v>
       </c>
       <c r="G4" t="n">
-        <v>0.3210878884957878</v>
+        <v>-0.03434251254026394</v>
       </c>
       <c r="H4" t="n">
-        <v>0.7060992795690617</v>
+        <v>0.7705075288837169</v>
       </c>
     </row>
     <row r="5">
@@ -2052,22 +2052,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.2227871776479093</v>
+        <v>0.2998108106936548</v>
       </c>
       <c r="D5" t="n">
-        <v>0.05659488653090335</v>
+        <v>0.1340917528631236</v>
       </c>
       <c r="E5" t="n">
-        <v>3.936524857705254</v>
+        <v>2.23586316303652</v>
       </c>
       <c r="F5" t="n">
-        <v>8.267006058786878e-05</v>
+        <v>0.02536073594032505</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1118632383382078</v>
+        <v>0.03699580445808692</v>
       </c>
       <c r="H5" t="n">
-        <v>0.3337111169576109</v>
+        <v>0.5626258169292226</v>
       </c>
     </row>
     <row r="6">
@@ -2082,22 +2082,22 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>-0.0233096983845467</v>
+        <v>-0.05897869106127263</v>
       </c>
       <c r="D6" t="n">
-        <v>0.03046167508096365</v>
+        <v>0.05145975489314585</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.7652139392397884</v>
+        <v>-1.146112941729698</v>
       </c>
       <c r="F6" t="n">
-        <v>0.4441441605977677</v>
+        <v>0.2517484233872033</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.08301348445199669</v>
+        <v>-0.1598379573050973</v>
       </c>
       <c r="H6" t="n">
-        <v>0.03639408768290329</v>
+        <v>0.04188057518255205</v>
       </c>
     </row>
   </sheetData>
@@ -2168,22 +2168,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>8.680144566698264</v>
+        <v>8.0059454933768</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6196822218451561</v>
+        <v>1.727728584819314</v>
       </c>
       <c r="E2" t="n">
-        <v>14.00741260714629</v>
+        <v>4.633798134568726</v>
       </c>
       <c r="F2" t="n">
-        <v>1.40428577088432e-44</v>
+        <v>3.590170950784332e-06</v>
       </c>
       <c r="G2" t="n">
-        <v>7.465589730021998</v>
+        <v>4.619659692070589</v>
       </c>
       <c r="H2" t="n">
-        <v>9.894699403374529</v>
+        <v>11.39223129468301</v>
       </c>
     </row>
     <row r="3">
@@ -2194,26 +2194,26 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tomatometer</t>
+          <t>PreRelease Tomatometer</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.002637922040813361</v>
+        <v>0.002981726155958417</v>
       </c>
       <c r="D3" t="n">
-        <v>0.001926508808132028</v>
+        <v>0.003790718081493591</v>
       </c>
       <c r="E3" t="n">
-        <v>1.369275878562491</v>
+        <v>0.7865861010649409</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1709130550900102</v>
+        <v>0.4315241981916041</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.001137965839024601</v>
+        <v>-0.004447944759313791</v>
       </c>
       <c r="H3" t="n">
-        <v>0.006413809920651322</v>
+        <v>0.01041139707123062</v>
       </c>
     </row>
     <row r="4">
@@ -2228,22 +2228,22 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.5630499931465542</v>
+        <v>0.5030335549775256</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1434122999237716</v>
+        <v>0.236966069301559</v>
       </c>
       <c r="E4" t="n">
-        <v>3.926092765026667</v>
+        <v>2.122808368557498</v>
       </c>
       <c r="F4" t="n">
-        <v>8.633686986284557e-05</v>
+        <v>0.03376991330007856</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2819670503559055</v>
+        <v>0.03858859358844741</v>
       </c>
       <c r="H4" t="n">
-        <v>0.844132935937203</v>
+        <v>0.9674785163666038</v>
       </c>
     </row>
     <row r="5">
@@ -2254,26 +2254,26 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tomatometer_Franchise</t>
+          <t>PreRelease_Tomatometer_Franchise</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.004782231557281379</v>
+        <v>0.00528669437274944</v>
       </c>
       <c r="D5" t="n">
-        <v>0.002436441722782443</v>
+        <v>0.004126750534538795</v>
       </c>
       <c r="E5" t="n">
-        <v>1.96279332789459</v>
+        <v>1.28107922407776</v>
       </c>
       <c r="F5" t="n">
-        <v>0.04967019340267143</v>
+        <v>0.2001658404619354</v>
       </c>
       <c r="G5" t="n">
-        <v>6.893530197067677e-06</v>
+        <v>-0.002801588048128013</v>
       </c>
       <c r="H5" t="n">
-        <v>0.00955756958436569</v>
+        <v>0.01337497679362689</v>
       </c>
     </row>
     <row r="6">
@@ -2288,22 +2288,22 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.4848454341477888</v>
+        <v>0.4318719216252473</v>
       </c>
       <c r="D6" t="n">
-        <v>0.08866771695739113</v>
+        <v>0.1518750378332205</v>
       </c>
       <c r="E6" t="n">
-        <v>5.468116816188908</v>
+        <v>2.843600421680234</v>
       </c>
       <c r="F6" t="n">
-        <v>4.548420949576293e-08</v>
+        <v>0.004460695011451415</v>
       </c>
       <c r="G6" t="n">
-        <v>0.3110599023199108</v>
+        <v>0.134202317321477</v>
       </c>
       <c r="H6" t="n">
-        <v>0.6586309659756668</v>
+        <v>0.7295415259290177</v>
       </c>
     </row>
     <row r="7">
@@ -2318,22 +2318,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.2861234194357755</v>
+        <v>0.3645278401438485</v>
       </c>
       <c r="D7" t="n">
-        <v>0.04822919067366088</v>
+        <v>0.1156816591655323</v>
       </c>
       <c r="E7" t="n">
-        <v>5.932577665916223</v>
+        <v>3.151129079349</v>
       </c>
       <c r="F7" t="n">
-        <v>2.982152432097517e-09</v>
+        <v>0.001626405955616877</v>
       </c>
       <c r="G7" t="n">
-        <v>0.1915959427118851</v>
+        <v>0.1377959545075674</v>
       </c>
       <c r="H7" t="n">
-        <v>0.3806508961596659</v>
+        <v>0.5912597257801296</v>
       </c>
     </row>
     <row r="8">
@@ -2348,22 +2348,22 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>-0.03310010926587099</v>
+        <v>-0.0491847134437994</v>
       </c>
       <c r="D8" t="n">
-        <v>0.02349970885674088</v>
+        <v>0.03524241507224854</v>
       </c>
       <c r="E8" t="n">
-        <v>-1.408532738326937</v>
+        <v>-1.395611320704569</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1589733798580949</v>
+        <v>0.1628315715249911</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.07915869227226005</v>
+        <v>-0.1182585777136181</v>
       </c>
       <c r="H8" t="n">
-        <v>0.01295847374051805</v>
+        <v>0.0198891508260193</v>
       </c>
     </row>
   </sheetData>

</xml_diff>